<commit_message>
correction des cases vides par région
</commit_message>
<xml_diff>
--- a/ressources.xlsx
+++ b/ressources.xlsx
@@ -5663,7 +5663,11 @@
           <t>04 73 82 71 00</t>
         </is>
       </c>
-      <c r="H100" s="12" t="n"/>
+      <c r="H100" s="12" t="inlineStr">
+        <is>
+          <t>http://www.ch-ambert.fr/</t>
+        </is>
+      </c>
       <c r="I100" s="12" t="inlineStr">
         <is>
           <t>direction@ch-ambert.fr</t>
@@ -8359,7 +8363,11 @@
           <t>04 71 78 40 00</t>
         </is>
       </c>
-      <c r="H152" s="12" t="n"/>
+      <c r="H152" s="12" t="inlineStr">
+        <is>
+          <t>https://www.ch-condat.fr/service/ehpad/</t>
+        </is>
+      </c>
       <c r="I152" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché à l'hôpital local de Condat</t>
@@ -8408,7 +8416,11 @@
           <t>04 71 67 33 33</t>
         </is>
       </c>
-      <c r="H153" s="12" t="n"/>
+      <c r="H153" s="12" t="inlineStr">
+        <is>
+          <t>http://www.ch-mauriac.fr</t>
+        </is>
+      </c>
       <c r="I153" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché au Centre hospitalier de Mauriac</t>
@@ -8555,7 +8567,11 @@
           <t>04 71 49 01 92</t>
         </is>
       </c>
-      <c r="H156" s="12" t="n"/>
+      <c r="H156" s="12" t="inlineStr">
+        <is>
+          <t>https://ehpadrogerjalenques.fr/</t>
+        </is>
+      </c>
       <c r="I156" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché à l'EHPAD Roger Jalenques</t>
@@ -8653,7 +8669,11 @@
           <t>04 71 46 56 56</t>
         </is>
       </c>
-      <c r="H158" s="12" t="n"/>
+      <c r="H158" s="12" t="inlineStr">
+        <is>
+          <t>http://www.ch-aurillac.fr</t>
+        </is>
+      </c>
       <c r="I158" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché au Centre hospitalier Henri Mondor</t>
@@ -9000,7 +9020,11 @@
           <t>04 71 01 10 00</t>
         </is>
       </c>
-      <c r="H165" s="12" t="n"/>
+      <c r="H165" s="12" t="inlineStr">
+        <is>
+          <t>http://www.hopital-craponne.fr</t>
+        </is>
+      </c>
       <c r="I165" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché au Centre hospitalier de Craponne</t>
@@ -9049,7 +9073,11 @@
           <t>04 71 03 42 90</t>
         </is>
       </c>
-      <c r="H166" s="12" t="n"/>
+      <c r="H166" s="12" t="inlineStr">
+        <is>
+          <t>http://www.foyermariegoy.com</t>
+        </is>
+      </c>
       <c r="I166" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché au Foyer de Personnes Âgées Marie Goy</t>
@@ -9098,7 +9126,11 @@
           <t>04 71 74 59 00</t>
         </is>
       </c>
-      <c r="H167" s="12" t="n"/>
+      <c r="H167" s="12" t="inlineStr">
+        <is>
+          <t>https://hoplangeac.fr</t>
+        </is>
+      </c>
       <c r="I167" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché au Centre hospitalier Pierre Gallice</t>
@@ -9147,7 +9179,11 @@
           <t>04 71 00 80 96</t>
         </is>
       </c>
-      <c r="H168" s="12" t="n"/>
+      <c r="H168" s="12" t="inlineStr">
+        <is>
+          <t>https://ehpad-pradelles.fr/</t>
+        </is>
+      </c>
       <c r="I168" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché à l'EHPAD Saint-Christophe</t>
@@ -9245,7 +9281,11 @@
           <t>04 71 66 61 17</t>
         </is>
       </c>
-      <c r="H170" s="12" t="n"/>
+      <c r="H170" s="12" t="inlineStr">
+        <is>
+          <t>https://residence-sigolene.fr</t>
+        </is>
+      </c>
       <c r="I170" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché à la Maison de Retraite Sigolène</t>
@@ -9343,7 +9383,11 @@
           <t>04 71 04 36 34</t>
         </is>
       </c>
-      <c r="H172" s="12" t="n"/>
+      <c r="H172" s="12" t="inlineStr">
+        <is>
+          <t>https://ehpad-st-joseph.fr</t>
+        </is>
+      </c>
       <c r="I172" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché à la Maison Saint-Joseph</t>
@@ -9441,7 +9485,11 @@
           <t>04 71 57 45 33</t>
         </is>
       </c>
-      <c r="H174" s="12" t="n"/>
+      <c r="H174" s="12" t="inlineStr">
+        <is>
+          <t>https://www.ahsm.fr/</t>
+        </is>
+      </c>
       <c r="I174" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché à l'EHPAD La Roseraie</t>
@@ -9543,7 +9591,11 @@
           <t>04 71 07 55 55</t>
         </is>
       </c>
-      <c r="H176" s="12" t="n"/>
+      <c r="H176" s="12" t="inlineStr">
+        <is>
+          <t>https://www.ahsm.fr/</t>
+        </is>
+      </c>
       <c r="I176" s="12" t="inlineStr">
         <is>
           <t>Accueil de jour Alzheimer, rattaché au Centre Hospitalier Sainte-Marie (unité Marie Pia)</t>
@@ -15038,7 +15090,11 @@
           <t>5 chemin des Alpins, 38000 Grenoble</t>
         </is>
       </c>
-      <c r="G281" s="11" t="n"/>
+      <c r="G281" s="11" t="inlineStr">
+        <is>
+          <t>04 76 23 11 16</t>
+        </is>
+      </c>
       <c r="H281" s="11" t="n"/>
       <c r="I281" s="11" t="n"/>
       <c r="J281" s="11" t="n">
@@ -15079,7 +15135,11 @@
           <t>1 rue Bévière, 38000 Grenoble</t>
         </is>
       </c>
-      <c r="G282" s="11" t="n"/>
+      <c r="G282" s="11" t="inlineStr">
+        <is>
+          <t>04 76 84 29 60</t>
+        </is>
+      </c>
       <c r="H282" s="11" t="n"/>
       <c r="I282" s="11" t="n"/>
       <c r="J282" s="11" t="n">
@@ -15115,9 +15175,21 @@
           <t>38 — Isère</t>
         </is>
       </c>
-      <c r="F283" s="11" t="n"/>
-      <c r="G283" s="11" t="n"/>
-      <c r="H283" s="11" t="n"/>
+      <c r="F283" s="11" t="inlineStr">
+        <is>
+          <t>13 rue Joseph Moutin, 38180 Seyssins</t>
+        </is>
+      </c>
+      <c r="G283" s="11" t="inlineStr">
+        <is>
+          <t>04 76 48 40 74</t>
+        </is>
+      </c>
+      <c r="H283" s="11" t="inlineStr">
+        <is>
+          <t>https://www.mutualiteisere.org/</t>
+        </is>
+      </c>
       <c r="I283" s="11" t="inlineStr">
         <is>
           <t>Adresse précise à confirmer auprès de l'établissement.</t>
@@ -15156,9 +15228,21 @@
           <t>38 — Isère</t>
         </is>
       </c>
-      <c r="F284" s="11" t="n"/>
-      <c r="G284" s="11" t="n"/>
-      <c r="H284" s="11" t="n"/>
+      <c r="F284" s="11" t="inlineStr">
+        <is>
+          <t>4 place Michel de Montaigne, 38320 Eybens</t>
+        </is>
+      </c>
+      <c r="G284" s="11" t="inlineStr">
+        <is>
+          <t>04 76 63 34 30</t>
+        </is>
+      </c>
+      <c r="H284" s="11" t="inlineStr">
+        <is>
+          <t>https://www.mutualiteisere.org/</t>
+        </is>
+      </c>
       <c r="I284" s="11" t="inlineStr">
         <is>
           <t>Adresse précise à confirmer auprès de l'établissement.</t>
@@ -15197,8 +15281,16 @@
           <t>38 — Isère</t>
         </is>
       </c>
-      <c r="F285" s="11" t="n"/>
-      <c r="G285" s="11" t="n"/>
+      <c r="F285" s="11" t="inlineStr">
+        <is>
+          <t>15 rue Eugène Charbonnier, 38600 Fontaine</t>
+        </is>
+      </c>
+      <c r="G285" s="11" t="inlineStr">
+        <is>
+          <t>04 38 03 10 50</t>
+        </is>
+      </c>
       <c r="H285" s="11" t="n"/>
       <c r="I285" s="11" t="inlineStr">
         <is>
@@ -15238,8 +15330,16 @@
           <t>38 — Isère</t>
         </is>
       </c>
-      <c r="F286" s="11" t="n"/>
-      <c r="G286" s="11" t="n"/>
+      <c r="F286" s="11" t="inlineStr">
+        <is>
+          <t>95 route de Chartreuse, 38700 Corenc</t>
+        </is>
+      </c>
+      <c r="G286" s="11" t="inlineStr">
+        <is>
+          <t>04 76 88 00 36</t>
+        </is>
+      </c>
       <c r="H286" s="11" t="n"/>
       <c r="I286" s="11" t="inlineStr">
         <is>
@@ -15279,8 +15379,16 @@
           <t>38 — Isère</t>
         </is>
       </c>
-      <c r="F287" s="11" t="n"/>
-      <c r="G287" s="11" t="n"/>
+      <c r="F287" s="11" t="inlineStr">
+        <is>
+          <t>360 rue de l'Eyrard, 38360 Noyarey</t>
+        </is>
+      </c>
+      <c r="G287" s="11" t="inlineStr">
+        <is>
+          <t>04 76 86 96 60</t>
+        </is>
+      </c>
       <c r="H287" s="11" t="n"/>
       <c r="I287" s="11" t="inlineStr">
         <is>
@@ -15320,8 +15428,16 @@
           <t>38 — Isère</t>
         </is>
       </c>
-      <c r="F288" s="11" t="n"/>
-      <c r="G288" s="11" t="n"/>
+      <c r="F288" s="11" t="inlineStr">
+        <is>
+          <t>14 rue Auguste et Edith Goirand, 38800 Le Pont-de-Claix</t>
+        </is>
+      </c>
+      <c r="G288" s="11" t="inlineStr">
+        <is>
+          <t>04 76 29 86 70</t>
+        </is>
+      </c>
       <c r="H288" s="11" t="n"/>
       <c r="I288" s="11" t="inlineStr">
         <is>
@@ -15361,8 +15477,16 @@
           <t>38 — Isère</t>
         </is>
       </c>
-      <c r="F289" s="11" t="n"/>
-      <c r="G289" s="11" t="n"/>
+      <c r="F289" s="11" t="inlineStr">
+        <is>
+          <t>6 rue du Gymnase, 38120 Saint-Égrève</t>
+        </is>
+      </c>
+      <c r="G289" s="11" t="inlineStr">
+        <is>
+          <t>04 76 75 44 55</t>
+        </is>
+      </c>
       <c r="H289" s="11" t="n"/>
       <c r="I289" s="11" t="inlineStr">
         <is>
@@ -15402,9 +15526,21 @@
           <t>38 — Isère</t>
         </is>
       </c>
-      <c r="F290" s="11" t="n"/>
-      <c r="G290" s="11" t="n"/>
-      <c r="H290" s="11" t="n"/>
+      <c r="F290" s="11" t="inlineStr">
+        <is>
+          <t>25 rue des Tillerets, 38450 Saint-Georges-de-Commiers</t>
+        </is>
+      </c>
+      <c r="G290" s="11" t="inlineStr">
+        <is>
+          <t>04 76 13 11 98</t>
+        </is>
+      </c>
+      <c r="H290" s="11" t="inlineStr">
+        <is>
+          <t>https://www.mutualiteisere.org/</t>
+        </is>
+      </c>
       <c r="I290" s="11" t="inlineStr">
         <is>
           <t>Adresse précise à confirmer auprès de l'établissement.</t>
@@ -15443,8 +15579,16 @@
           <t>38 — Isère</t>
         </is>
       </c>
-      <c r="F291" s="11" t="n"/>
-      <c r="G291" s="11" t="n"/>
+      <c r="F291" s="11" t="inlineStr">
+        <is>
+          <t>9 chemin du Mas de Saint Germain, 38700 La Tronche</t>
+        </is>
+      </c>
+      <c r="G291" s="11" t="inlineStr">
+        <is>
+          <t>04 76 41 63 30</t>
+        </is>
+      </c>
       <c r="H291" s="11" t="n"/>
       <c r="I291" s="11" t="inlineStr">
         <is>
@@ -20516,7 +20660,11 @@
           <t>53 chemin de Parenty, 69250 Neuville-sur-Saône</t>
         </is>
       </c>
-      <c r="G395" s="11" t="n"/>
+      <c r="G395" s="11" t="inlineStr">
+        <is>
+          <t>04 72 00 10 35</t>
+        </is>
+      </c>
       <c r="H395" s="11" t="n"/>
       <c r="I395" s="11" t="n"/>
       <c r="J395" s="11" t="n">
@@ -20601,8 +20749,16 @@
           <t>69 — Rhône</t>
         </is>
       </c>
-      <c r="F397" s="11" t="n"/>
-      <c r="G397" s="11" t="n"/>
+      <c r="F397" s="11" t="inlineStr">
+        <is>
+          <t>41 rue André Sabatier, 69520 Grigny</t>
+        </is>
+      </c>
+      <c r="G397" s="11" t="inlineStr">
+        <is>
+          <t>04 72 24 16 56</t>
+        </is>
+      </c>
       <c r="H397" s="11" t="n"/>
       <c r="I397" s="11" t="n"/>
       <c r="J397" s="11" t="n">
@@ -20638,8 +20794,16 @@
           <t>69 — Rhône</t>
         </is>
       </c>
-      <c r="F398" s="11" t="n"/>
-      <c r="G398" s="11" t="n"/>
+      <c r="F398" s="11" t="inlineStr">
+        <is>
+          <t>15 route de Champagne, 69130 Écully</t>
+        </is>
+      </c>
+      <c r="G398" s="11" t="inlineStr">
+        <is>
+          <t>04 78 33 56 42</t>
+        </is>
+      </c>
       <c r="H398" s="11" t="n"/>
       <c r="I398" s="11" t="n"/>
       <c r="J398" s="11" t="n">
@@ -20675,8 +20839,16 @@
           <t>69 — Rhône</t>
         </is>
       </c>
-      <c r="F399" s="11" t="n"/>
-      <c r="G399" s="11" t="n"/>
+      <c r="F399" s="11" t="inlineStr">
+        <is>
+          <t>19 rue du Capitaine Ferber, 69300 Caluire-et-Cuire</t>
+        </is>
+      </c>
+      <c r="G399" s="11" t="inlineStr">
+        <is>
+          <t>04 78 29 34 98</t>
+        </is>
+      </c>
       <c r="H399" s="11" t="n"/>
       <c r="I399" s="11" t="n"/>
       <c r="J399" s="11" t="n">
@@ -20712,8 +20884,16 @@
           <t>69 — Rhône</t>
         </is>
       </c>
-      <c r="F400" s="11" t="n"/>
-      <c r="G400" s="11" t="n"/>
+      <c r="F400" s="11" t="inlineStr">
+        <is>
+          <t>Place de l'Église, 69670 Vaugneray</t>
+        </is>
+      </c>
+      <c r="G400" s="11" t="inlineStr">
+        <is>
+          <t>04 78 16 80 80</t>
+        </is>
+      </c>
       <c r="H400" s="11" t="n"/>
       <c r="I400" s="11" t="n"/>
       <c r="J400" s="11" t="n">
@@ -20798,9 +20978,21 @@
           <t>69 — Rhône</t>
         </is>
       </c>
-      <c r="F402" s="11" t="n"/>
-      <c r="G402" s="11" t="n"/>
-      <c r="H402" s="11" t="n"/>
+      <c r="F402" s="11" t="inlineStr">
+        <is>
+          <t>34 rue Henri Lebrun, 69330 Meyzieu</t>
+        </is>
+      </c>
+      <c r="G402" s="11" t="inlineStr">
+        <is>
+          <t>04 78 31 09 09</t>
+        </is>
+      </c>
+      <c r="H402" s="11" t="inlineStr">
+        <is>
+          <t>https://www.margueritemeyzieu.com/</t>
+        </is>
+      </c>
       <c r="I402" s="11" t="n"/>
       <c r="J402" s="11" t="n">
         <v>45.7686</v>

</xml_diff>